<commit_message>
MD-neutral reference form: the multiple district is stamped from config
The reference workbook no longer carries any MD 112 or Belgium value:
V1 (country), AB1 (MD), AE67, AH78, AH85 and F104 are blank and the
filler stamps them at load from the new MD and MD_COUNTRY constants in
districts_data.js, alongside the district letter and coordinator. Every
"112" hard-coded in the code (file names, labels, e-mail subjects,
tracker badges and CSV, admin paths) now derives from MD, so a national
fork gets its own multiple district by editing districts_data.js only.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01FkcJjMbMkr4Y9DdTdEC2Q4
</commit_message>
<xml_diff>
--- a/Application_form_2026_MD112.xlsx
+++ b/Application_form_2026_MD112.xlsx
@@ -3419,9 +3419,7 @@
       <c r="U1" s="67" t="s">
         <v>24</v>
       </c>
-      <c r="V1" s="205" t="s">
-        <v>138</v>
-      </c>
+      <c r="V1" s="205"/>
       <c r="W1" s="205"/>
       <c r="X1" s="205"/>
       <c r="Y1" s="67" t="s">
@@ -3431,9 +3429,7 @@
         <v>40</v>
       </c>
       <c r="AA1" s="206"/>
-      <c r="AB1" s="207" t="s">
-        <v>139</v>
-      </c>
+      <c r="AB1" s="207"/>
       <c r="AC1" s="208"/>
       <c r="AD1" s="123" t="s">
         <v>63</v>
@@ -6496,9 +6492,7 @@
       <c r="AB67" s="88"/>
       <c r="AC67" s="88"/>
       <c r="AD67" s="89"/>
-      <c r="AE67" s="170" t="s">
-        <v>146</v>
-      </c>
+      <c r="AE67" s="170"/>
       <c r="AF67" s="171"/>
       <c r="AG67" s="171"/>
       <c r="AH67" s="171"/>
@@ -6954,11 +6948,7 @@
       <c r="AE78" s="80"/>
       <c r="AF78" s="80"/>
       <c r="AG78" s="80"/>
-      <c r="AH78" s="170" t="inlineStr">
-        <is>
-          <t>112</t>
-        </is>
-      </c>
+      <c r="AH78" s="170"/>
       <c r="AI78" s="171"/>
       <c r="AJ78" s="171"/>
       <c r="AK78" s="172"/>
@@ -7244,9 +7234,7 @@
       <c r="AE85" s="80"/>
       <c r="AF85" s="80"/>
       <c r="AG85" s="80"/>
-      <c r="AH85" s="348" t="s">
-        <v>146</v>
-      </c>
+      <c r="AH85" s="348"/>
       <c r="AI85" s="348"/>
       <c r="AJ85" s="348"/>
       <c r="AK85" s="348"/>
@@ -7995,9 +7983,7 @@
       <c r="C104" s="188"/>
       <c r="D104" s="188"/>
       <c r="E104" s="189"/>
-      <c r="F104" s="281" t="s">
-        <v>147</v>
-      </c>
+      <c r="F104" s="281"/>
       <c r="G104" s="191"/>
       <c r="H104" s="191"/>
       <c r="I104" s="191"/>

</xml_diff>